<commit_message>
Standardize CargoBay mass attribute and misc fixes
Replace uses of .cargo.mass_properties.mass with .mass_properties.mass across vehicle, tutorial, and docs files to match Cargo_Bay API. Add Vref_VS_ratio attribute to Vehicle. Remove strict mission type checks / tidy docstrings in compute_load_and_trim_diagram and compute_noise_certification_metrics. Pass show_figure=False to plot_3d_vehicle in battery_electric_aircraft_test. Enable many verification modules in the automatic regression list and update related regression Excel blobs. These changes align code with updated component interfaces and improve test coverage/behavior.
</commit_message>
<xml_diff>
--- a/VnV/test_automatic_regression_weight_breakdown.xlsx
+++ b/VnV/test_automatic_regression_weight_breakdown.xlsx
@@ -1692,16 +1692,16 @@
         <v>92601.33</v>
       </c>
       <c r="D2" t="n">
-        <v>400246.37</v>
+        <v>399902.95</v>
       </c>
       <c r="E2" t="n">
-        <v>459704.97</v>
+        <v>459361.55</v>
       </c>
       <c r="F2" t="n">
-        <v>-169322.86</v>
+        <v>-169246.81</v>
       </c>
       <c r="G2" t="n">
-        <v>-77026.55</v>
+        <v>-76991.95</v>
       </c>
       <c r="H2" t="n">
         <v>-34106.32</v>
@@ -1720,16 +1720,16 @@
         <v>10172.2</v>
       </c>
       <c r="D3" t="n">
-        <v>43832.78</v>
+        <v>43795.2</v>
       </c>
       <c r="E3" t="n">
-        <v>50338.68</v>
+        <v>50301.1</v>
       </c>
       <c r="F3" t="n">
-        <v>-18527.13</v>
+        <v>-18518.81</v>
       </c>
       <c r="G3" t="n">
-        <v>-8428.17</v>
+        <v>-8424.379999999999</v>
       </c>
       <c r="H3" t="n">
         <v>-3731.88</v>
@@ -1748,16 +1748,16 @@
         <v>92601.33</v>
       </c>
       <c r="D4" t="n">
-        <v>400246.37</v>
+        <v>399902.95</v>
       </c>
       <c r="E4" t="n">
-        <v>459704.97</v>
+        <v>459361.55</v>
       </c>
       <c r="F4" t="n">
-        <v>169322.86</v>
+        <v>169246.81</v>
       </c>
       <c r="G4" t="n">
-        <v>-77026.55</v>
+        <v>-76991.95</v>
       </c>
       <c r="H4" t="n">
         <v>34106.32</v>
@@ -1776,16 +1776,16 @@
         <v>10172.2</v>
       </c>
       <c r="D5" t="n">
-        <v>43832.78</v>
+        <v>43795.2</v>
       </c>
       <c r="E5" t="n">
-        <v>50338.68</v>
+        <v>50301.1</v>
       </c>
       <c r="F5" t="n">
-        <v>18527.13</v>
+        <v>18518.81</v>
       </c>
       <c r="G5" t="n">
-        <v>-8428.17</v>
+        <v>-8424.379999999999</v>
       </c>
       <c r="H5" t="n">
         <v>3731.88</v>
@@ -1804,16 +1804,16 @@
         <v>14750.29</v>
       </c>
       <c r="D6" t="n">
-        <v>18087.2</v>
+        <v>18062.91</v>
       </c>
       <c r="E6" t="n">
-        <v>32591.6</v>
+        <v>32567.32</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>968.01</v>
+        <v>966.47</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -1832,16 +1832,16 @@
         <v>95036.99000000001</v>
       </c>
       <c r="D7" t="n">
-        <v>2922.94</v>
+        <v>2936.52</v>
       </c>
       <c r="E7" t="n">
-        <v>96628.27</v>
+        <v>96641.85000000001</v>
       </c>
       <c r="F7" t="n">
-        <v>12754.22</v>
+        <v>12800.97</v>
       </c>
       <c r="G7" t="n">
-        <v>689.54</v>
+        <v>692.0599999999999</v>
       </c>
       <c r="H7" t="n">
         <v>-4757.65</v>
@@ -1860,16 +1860,16 @@
         <v>101417.27</v>
       </c>
       <c r="D8" t="n">
-        <v>8546.77</v>
+        <v>8562.299999999999</v>
       </c>
       <c r="E8" t="n">
-        <v>108946.92</v>
+        <v>108962.45</v>
       </c>
       <c r="F8" t="n">
-        <v>14593.87</v>
+        <v>14647.35</v>
       </c>
       <c r="G8" t="n">
-        <v>788.99</v>
+        <v>791.89</v>
       </c>
       <c r="H8" t="n">
         <v>-5443.89</v>
@@ -1888,16 +1888,16 @@
         <v>90768.92</v>
       </c>
       <c r="D9" t="n">
-        <v>1122.7</v>
+        <v>1116.87</v>
       </c>
       <c r="E9" t="n">
-        <v>91053.77</v>
+        <v>91047.94</v>
       </c>
       <c r="F9" t="n">
-        <v>-6570.3</v>
+        <v>-6531.52</v>
       </c>
       <c r="G9" t="n">
-        <v>-323.05</v>
+        <v>-321.15</v>
       </c>
       <c r="H9" t="n">
         <v>-4283.83</v>
@@ -1916,16 +1916,16 @@
         <v>86732.2</v>
       </c>
       <c r="D10" t="n">
-        <v>3294.98</v>
+        <v>3289.2</v>
       </c>
       <c r="E10" t="n">
-        <v>89424.39</v>
+        <v>89418.61</v>
       </c>
       <c r="F10" t="n">
-        <v>-6510.97</v>
+        <v>-6472.54</v>
       </c>
       <c r="G10" t="n">
-        <v>-320.14</v>
+        <v>-318.25</v>
       </c>
       <c r="H10" t="n">
         <v>-4245.15</v>
@@ -1944,16 +1944,16 @@
         <v>2045.64</v>
       </c>
       <c r="D11" t="n">
-        <v>106232.82</v>
+        <v>106083.69</v>
       </c>
       <c r="E11" t="n">
-        <v>104187.17</v>
+        <v>104038.05</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>14598.96</v>
+        <v>14588.51</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -1972,16 +1972,16 @@
         <v>2161.93</v>
       </c>
       <c r="D12" t="n">
-        <v>96132.41</v>
+        <v>95997.53999999999</v>
       </c>
       <c r="E12" t="n">
-        <v>94501.78999999999</v>
+        <v>94366.92</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>13203.12</v>
+        <v>13193.67</v>
       </c>
       <c r="H12" t="n">
         <v>-0</v>
@@ -2000,16 +2000,16 @@
         <v>99.23</v>
       </c>
       <c r="D13" t="n">
-        <v>8183.57</v>
+        <v>8176.31</v>
       </c>
       <c r="E13" t="n">
-        <v>8262.299999999999</v>
+        <v>8255.040000000001</v>
       </c>
       <c r="F13" t="n">
-        <v>-852.8</v>
+        <v>-852.4299999999999</v>
       </c>
       <c r="G13" t="n">
-        <v>289.43</v>
+        <v>289.3</v>
       </c>
       <c r="H13" t="n">
         <v>30.2</v>
@@ -2028,16 +2028,16 @@
         <v>99.23</v>
       </c>
       <c r="D14" t="n">
-        <v>8183.57</v>
+        <v>8176.31</v>
       </c>
       <c r="E14" t="n">
-        <v>8262.299999999999</v>
+        <v>8255.040000000001</v>
       </c>
       <c r="F14" t="n">
-        <v>852.8</v>
+        <v>852.4299999999999</v>
       </c>
       <c r="G14" t="n">
-        <v>289.43</v>
+        <v>289.3</v>
       </c>
       <c r="H14" t="n">
         <v>-30.2</v>
@@ -2056,16 +2056,16 @@
         <v>10.25</v>
       </c>
       <c r="D15" t="n">
-        <v>8183.57</v>
+        <v>8176.31</v>
       </c>
       <c r="E15" t="n">
-        <v>8173.32</v>
+        <v>8166.06</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>289.43</v>
+        <v>289.3</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -2084,16 +2084,16 @@
         <v>99.23</v>
       </c>
       <c r="D16" t="n">
-        <v>8183.57</v>
+        <v>8176.31</v>
       </c>
       <c r="E16" t="n">
-        <v>8262.299999999999</v>
+        <v>8255.040000000001</v>
       </c>
       <c r="F16" t="n">
-        <v>-852.8</v>
+        <v>-852.4299999999999</v>
       </c>
       <c r="G16" t="n">
-        <v>289.43</v>
+        <v>289.3</v>
       </c>
       <c r="H16" t="n">
         <v>30.2</v>
@@ -2112,16 +2112,16 @@
         <v>1130090.96</v>
       </c>
       <c r="D17" t="n">
-        <v>434603.11</v>
+        <v>434200.33</v>
       </c>
       <c r="E17" t="n">
-        <v>1547444.35</v>
+        <v>1547041.57</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>-27242.7</v>
+        <v>-27218.81</v>
       </c>
       <c r="H17" t="n">
         <v>-0</v>
@@ -2140,16 +2140,16 @@
         <v>249769.84</v>
       </c>
       <c r="D18" t="n">
-        <v>1191349.78</v>
+        <v>1192249.06</v>
       </c>
       <c r="E18" t="n">
-        <v>1352890.25</v>
+        <v>1353789.54</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>-18115.57</v>
+        <v>-18127.28</v>
       </c>
       <c r="H18" t="n">
         <v>0</v>
@@ -2168,16 +2168,16 @@
         <v>65087.24</v>
       </c>
       <c r="D19" t="n">
-        <v>465050</v>
+        <v>464647.76</v>
       </c>
       <c r="E19" t="n">
-        <v>519939.15</v>
+        <v>519536.91</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>3450.29</v>
+        <v>3448.7</v>
       </c>
       <c r="H19" t="n">
         <v>-0</v>
@@ -2196,16 +2196,16 @@
         <v>87353.55</v>
       </c>
       <c r="D20" t="n">
-        <v>400258.09</v>
+        <v>397792.4</v>
       </c>
       <c r="E20" t="n">
-        <v>312917.37</v>
+        <v>310451.68</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>-8145.7</v>
+        <v>-8010.44</v>
       </c>
       <c r="H20" t="n">
         <v>-0</v>
@@ -2224,16 +2224,16 @@
         <v>160650.21</v>
       </c>
       <c r="D21" t="n">
-        <v>683565.09</v>
+        <v>683861.09</v>
       </c>
       <c r="E21" t="n">
-        <v>522938.47</v>
+        <v>523234.47</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>-11780.24</v>
+        <v>-11800.7</v>
       </c>
       <c r="H21" t="n">
         <v>-0</v>
@@ -2252,16 +2252,16 @@
         <v>15911.48</v>
       </c>
       <c r="D22" t="n">
-        <v>59052.33</v>
+        <v>59011.63</v>
       </c>
       <c r="E22" t="n">
-        <v>74840.62</v>
+        <v>74799.92</v>
       </c>
       <c r="F22" t="n">
-        <v>-30577.71</v>
+        <v>-30567.16</v>
       </c>
       <c r="G22" t="n">
-        <v>-1906.18</v>
+        <v>-1905.52</v>
       </c>
       <c r="H22" t="n">
         <v>-988.0599999999999</v>
@@ -2280,16 +2280,16 @@
         <v>145.09</v>
       </c>
       <c r="D23" t="n">
-        <v>372270.53</v>
+        <v>372455.03</v>
       </c>
       <c r="E23" t="n">
-        <v>372125.44</v>
+        <v>372309.94</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>-7347.96</v>
+        <v>-7349.79</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
@@ -2308,16 +2308,16 @@
         <v>335.95</v>
       </c>
       <c r="D24" t="n">
-        <v>2656.19</v>
+        <v>2678.4</v>
       </c>
       <c r="E24" t="n">
-        <v>2320.24</v>
+        <v>2342.46</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>-882.88</v>
+        <v>-887.1</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
@@ -2336,16 +2336,16 @@
         <v>27.16</v>
       </c>
       <c r="D25" t="n">
-        <v>15504.67</v>
+        <v>15488.39</v>
       </c>
       <c r="E25" t="n">
-        <v>15477.51</v>
+        <v>15461.23</v>
       </c>
       <c r="F25" t="n">
         <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>648.35</v>
+        <v>648.01</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -2364,16 +2364,16 @@
         <v>970.36</v>
       </c>
       <c r="D26" t="n">
-        <v>15504.67</v>
+        <v>15488.39</v>
       </c>
       <c r="E26" t="n">
-        <v>16420.71</v>
+        <v>16404.43</v>
       </c>
       <c r="F26" t="n">
-        <v>3820.78</v>
+        <v>3818.77</v>
       </c>
       <c r="G26" t="n">
-        <v>648.35</v>
+        <v>648.01</v>
       </c>
       <c r="H26" t="n">
         <v>-160.05</v>
@@ -2392,16 +2392,16 @@
         <v>970.36</v>
       </c>
       <c r="D27" t="n">
-        <v>15504.67</v>
+        <v>15488.39</v>
       </c>
       <c r="E27" t="n">
-        <v>16420.71</v>
+        <v>16404.43</v>
       </c>
       <c r="F27" t="n">
-        <v>-3820.78</v>
+        <v>-3818.77</v>
       </c>
       <c r="G27" t="n">
-        <v>648.35</v>
+        <v>648.01</v>
       </c>
       <c r="H27" t="n">
         <v>160.05</v>
@@ -2420,16 +2420,16 @@
         <v>346.6</v>
       </c>
       <c r="D28" t="n">
-        <v>382497.33</v>
+        <v>382786.32</v>
       </c>
       <c r="E28" t="n">
-        <v>382150.74</v>
+        <v>382439.72</v>
       </c>
       <c r="F28" t="n">
         <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>-11508.78</v>
+        <v>-11513.13</v>
       </c>
       <c r="H28" t="n">
         <v>0</v>
@@ -2448,16 +2448,16 @@
         <v>210.66</v>
       </c>
       <c r="D29" t="n">
-        <v>66630.55</v>
+        <v>66536.67</v>
       </c>
       <c r="E29" t="n">
-        <v>66419.89</v>
+        <v>66326.02</v>
       </c>
       <c r="F29" t="n">
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>3740.55</v>
+        <v>3737.91</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
@@ -2476,16 +2476,16 @@
         <v>181.58</v>
       </c>
       <c r="D30" t="n">
-        <v>200382.8</v>
+        <v>200534.2</v>
       </c>
       <c r="E30" t="n">
-        <v>200201.22</v>
+        <v>200352.62</v>
       </c>
       <c r="F30" t="n">
         <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>-6029.22</v>
+        <v>-6031.5</v>
       </c>
       <c r="H30" t="n">
         <v>0</v>
@@ -2504,16 +2504,16 @@
         <v>49.75</v>
       </c>
       <c r="D31" t="n">
-        <v>127657.77</v>
+        <v>127721.03</v>
       </c>
       <c r="E31" t="n">
-        <v>127608.01</v>
+        <v>127671.28</v>
       </c>
       <c r="F31" t="n">
         <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>-2519.74</v>
+        <v>-2520.36</v>
       </c>
       <c r="H31" t="n">
         <v>0</v>
@@ -2532,16 +2532,16 @@
         <v>2600.06</v>
       </c>
       <c r="D32" t="n">
-        <v>55950.78</v>
+        <v>55816.21</v>
       </c>
       <c r="E32" t="n">
-        <v>55976.54</v>
+        <v>55841.97</v>
       </c>
       <c r="F32" t="n">
         <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>5363.65</v>
+        <v>5356.95</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
@@ -2560,16 +2560,16 @@
         <v>168.95</v>
       </c>
       <c r="D33" t="n">
-        <v>73616.97</v>
+        <v>73669.63</v>
       </c>
       <c r="E33" t="n">
-        <v>73556.78</v>
+        <v>73609.45</v>
       </c>
       <c r="F33" t="n">
         <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>-2097.53</v>
+        <v>-2098.28</v>
       </c>
       <c r="H33" t="n">
         <v>0</v>
@@ -2588,16 +2588,16 @@
         <v>5318.39</v>
       </c>
       <c r="D34" t="n">
-        <v>35009.86</v>
+        <v>35044.69</v>
       </c>
       <c r="E34" t="n">
-        <v>32977.94</v>
+        <v>33012.77</v>
       </c>
       <c r="F34" t="n">
         <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>-5469.43</v>
+        <v>-5480.08</v>
       </c>
       <c r="H34" t="n">
         <v>0</v>
@@ -2616,16 +2616,16 @@
         <v>6388.66</v>
       </c>
       <c r="D35" t="n">
-        <v>6929.44</v>
+        <v>6933.86</v>
       </c>
       <c r="E35" t="n">
-        <v>10349.7</v>
+        <v>10354.13</v>
       </c>
       <c r="F35" t="n">
-        <v>-1295.58</v>
+        <v>-1303.61</v>
       </c>
       <c r="G35" t="n">
-        <v>-694.11</v>
+        <v>-698.41</v>
       </c>
       <c r="H35" t="n">
         <v>-2524.49</v>
@@ -2644,16 +2644,16 @@
         <v>6388.66</v>
       </c>
       <c r="D36" t="n">
-        <v>6929.44</v>
+        <v>6933.86</v>
       </c>
       <c r="E36" t="n">
-        <v>10349.7</v>
+        <v>10354.13</v>
       </c>
       <c r="F36" t="n">
-        <v>1295.58</v>
+        <v>1303.61</v>
       </c>
       <c r="G36" t="n">
-        <v>-694.11</v>
+        <v>-698.41</v>
       </c>
       <c r="H36" t="n">
         <v>2524.49</v>
@@ -2672,16 +2672,16 @@
         <v>2331733.75</v>
       </c>
       <c r="D37" t="n">
-        <v>5768156.41</v>
+        <v>5765487.92</v>
       </c>
       <c r="E37" t="n">
-        <v>7383706.77</v>
+        <v>7381038.28</v>
       </c>
       <c r="F37" t="n">
-        <v>-17163.69</v>
+        <v>-16975.33</v>
       </c>
       <c r="G37" t="n">
-        <v>-230080.92</v>
+        <v>-229934.52</v>
       </c>
       <c r="H37" t="n">
         <v>-19688.38</v>

</xml_diff>